<commit_message>
feat(run): complete G5 holdings and G6 nodes
</commit_message>
<xml_diff>
--- a/DataTables/Datas/__tables__.xlsx
+++ b/DataTables/Datas/__tables__.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R631dc41231ea4737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6c2c309b2c14424d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -901,6 +901,60 @@
       <x:c r="J12"/>
       <x:c r="K12"/>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13"/>
+      <x:c r="B13" t="str">
+        <x:v>run.TbRelic</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>run.Relic</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>run.relic.xlsx</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="H13"/>
+      <x:c r="I13" t="str">
+        <x:v>Run relic static template</x:v>
+      </x:c>
+      <x:c r="J13"/>
+      <x:c r="K13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14"/>
+      <x:c r="B14" t="str">
+        <x:v>run.TbPotion</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>run.Potion</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>run.potion.xlsx</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="H14"/>
+      <x:c r="I14" t="str">
+        <x:v>Run potion static template</x:v>
+      </x:c>
+      <x:c r="J14"/>
+      <x:c r="K14"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>